<commit_message>
Data updates and README note for AbTeC team
- Reparse timeline-data.js from updated xlsx (AbInt moved to Program)
- README: add taxonomy validation note for Nancy/AbTeC team

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/timeline-data/timeline-data.xlsx
+++ b/data/timeline-data/timeline-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasonlocal/Documents/Coding-Experiments/Timeline/Timeline-JEL/data/timeline-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64D083DF-5DC8-E64E-94FA-40E048C29609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CE4543-A537-0C47-9D4B-DD45B0784991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4600" yWindow="500" windowWidth="33700" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -299,7 +299,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5017" uniqueCount="2142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5017" uniqueCount="2141">
   <si>
     <t>Year</t>
   </si>
@@ -6781,9 +6781,6 @@
   </si>
   <si>
     <t>Integrations</t>
-  </si>
-  <si>
-    <t>Epistemological Foundations</t>
   </si>
   <si>
     <t>2023</t>
@@ -8378,7 +8375,7 @@
         <v>26</v>
       </c>
       <c r="S2" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T2" s="7" t="s">
         <v>28</v>
@@ -8414,39 +8411,39 @@
       <c r="H3" s="10"/>
       <c r="I3" s="9"/>
       <c r="J3" s="115" t="s">
+        <v>2136</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>2138</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>2139</v>
+      </c>
+      <c r="M3" s="14" t="s">
         <v>2137</v>
-      </c>
-      <c r="K3" s="12" t="s">
-        <v>2139</v>
-      </c>
-      <c r="L3" s="13" t="s">
-        <v>2140</v>
-      </c>
-      <c r="M3" s="14" t="s">
-        <v>2138</v>
       </c>
       <c r="N3" s="7"/>
       <c r="O3" s="7"/>
       <c r="P3" s="7" t="s">
-        <v>2141</v>
+        <v>2140</v>
       </c>
       <c r="Q3" s="7" t="s">
         <v>2132</v>
       </c>
       <c r="R3" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="S3" s="7" t="s">
         <v>2133</v>
       </c>
-      <c r="S3" s="7" t="s">
+      <c r="T3" s="7" t="s">
         <v>2134</v>
-      </c>
-      <c r="T3" s="7" t="s">
-        <v>2135</v>
       </c>
       <c r="U3" s="15" t="s">
         <v>38</v>
       </c>
       <c r="V3" s="15" t="s">
-        <v>2136</v>
+        <v>2135</v>
       </c>
       <c r="W3" s="15"/>
       <c r="X3" s="16" t="s">

</xml_diff>